<commit_message>
1.7.2 and first stage of code refactoring
</commit_message>
<xml_diff>
--- a/Templates/OSX-100 Single Mode COC Template 1.xlsx
+++ b/Templates/OSX-100 Single Mode COC Template 1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Austin\Documents\Python Stuff\ILM Python Testing\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9BAE208-751B-4412-A031-8D7F167B89E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D7969B2-1686-415E-8352-90AA72D5038A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-5220" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{2EE93342-3441-4D7E-B34D-C071F052B887}"/>
   </bookViews>
@@ -142,10 +142,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yymmdd"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
   <fonts count="45" x14ac:knownFonts="1">
     <font>
@@ -954,81 +953,78 @@
     <xf numFmtId="0" fontId="38" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="39" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="42" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="42" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -1040,6 +1036,9 @@
     </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="41" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="39" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="53">
@@ -1699,28 +1698,28 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="53" t="s">
+      <c r="A2" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="53"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="53"/>
-      <c r="F2" s="53"/>
-      <c r="G2" s="53"/>
-      <c r="H2" s="53"/>
-      <c r="I2" s="53"/>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="52"/>
     </row>
     <row r="4" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="54" t="s">
+      <c r="B4" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54"/>
-      <c r="E4" s="54"/>
+      <c r="C4" s="53"/>
+      <c r="D4" s="53"/>
+      <c r="E4" s="53"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="4"/>
@@ -1729,19 +1728,19 @@
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="54">
+      <c r="B6" s="53">
         <v>15367</v>
       </c>
-      <c r="C6" s="54"/>
+      <c r="C6" s="53"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="55">
+      <c r="B7" s="54">
         <v>44165</v>
       </c>
-      <c r="C7" s="55"/>
+      <c r="C7" s="54"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
@@ -1930,17 +1929,17 @@
       <c r="B35"/>
     </row>
     <row r="36" spans="1:9" s="19" customFormat="1" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="56" t="s">
+      <c r="A36" s="55" t="s">
         <v>16</v>
       </c>
-      <c r="B36" s="56"/>
-      <c r="C36" s="56"/>
-      <c r="D36" s="56"/>
-      <c r="E36" s="56"/>
-      <c r="F36" s="56"/>
-      <c r="G36" s="56"/>
-      <c r="H36" s="56"/>
-      <c r="I36" s="56"/>
+      <c r="B36" s="55"/>
+      <c r="C36" s="55"/>
+      <c r="D36" s="55"/>
+      <c r="E36" s="55"/>
+      <c r="F36" s="55"/>
+      <c r="G36" s="55"/>
+      <c r="H36" s="55"/>
+      <c r="I36" s="55"/>
     </row>
     <row r="37" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="46" spans="1:9" ht="78" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1973,14 +1972,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:8" ht="84.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B1" s="50" t="s">
+      <c r="B1" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
-      <c r="F1" s="50"/>
-      <c r="G1" s="50"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
     </row>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="21"/>
@@ -1991,14 +1990,14 @@
       <c r="G2" s="21"/>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B3" s="51" t="s">
+      <c r="B3" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="51"/>
-      <c r="D3" s="51" t="s">
+      <c r="C3" s="29"/>
+      <c r="D3" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="51"/>
+      <c r="E3" s="29"/>
       <c r="F3" s="22" t="s">
         <v>20</v>
       </c>
@@ -2007,10 +2006,10 @@
       </c>
     </row>
     <row r="4" spans="2:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="52"/>
-      <c r="C4" s="52"/>
-      <c r="D4" s="52"/>
-      <c r="E4" s="52"/>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
       <c r="F4" s="23"/>
       <c r="G4" s="24"/>
     </row>
@@ -2024,62 +2023,62 @@
       <c r="H5" s="25"/>
     </row>
     <row r="6" spans="2:8" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="40"/>
-      <c r="C6" s="41"/>
-      <c r="D6" s="42" t="s">
+      <c r="B6" s="31"/>
+      <c r="C6" s="32"/>
+      <c r="D6" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="E6" s="42"/>
-      <c r="F6" s="42"/>
-      <c r="G6" s="42"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
       <c r="H6" s="25"/>
     </row>
     <row r="7" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="48" t="s">
+      <c r="B7" s="34" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="49"/>
-      <c r="D7" s="42" t="s">
+      <c r="C7" s="35"/>
+      <c r="D7" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="42"/>
-      <c r="F7" s="42" t="s">
+      <c r="E7" s="33"/>
+      <c r="F7" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="G7" s="42"/>
+      <c r="G7" s="33"/>
       <c r="H7" s="25"/>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="46" t="s">
+      <c r="B8" s="36" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="46"/>
-      <c r="D8" s="47" t="s">
+      <c r="C8" s="36"/>
+      <c r="D8" s="37" t="s">
         <v>27</v>
       </c>
-      <c r="E8" s="47"/>
-      <c r="F8" s="47" t="s">
+      <c r="E8" s="37"/>
+      <c r="F8" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="G8" s="47"/>
+      <c r="G8" s="37"/>
       <c r="H8" s="25"/>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="46"/>
-      <c r="C9" s="46"/>
-      <c r="D9" s="47" t="s">
+      <c r="B9" s="36"/>
+      <c r="C9" s="36"/>
+      <c r="D9" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="47"/>
-      <c r="F9" s="47" t="s">
+      <c r="E9" s="37"/>
+      <c r="F9" s="37" t="s">
         <v>32</v>
       </c>
-      <c r="G9" s="47"/>
+      <c r="G9" s="37"/>
       <c r="H9" s="25"/>
     </row>
     <row r="10" spans="2:8" ht="10.199999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="46"/>
-      <c r="C10" s="46"/>
+      <c r="B10" s="36"/>
+      <c r="C10" s="36"/>
       <c r="D10" s="26" t="s">
         <v>29</v>
       </c>
@@ -2095,472 +2094,472 @@
       <c r="H10" s="25"/>
     </row>
     <row r="11" spans="2:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="34">
+      <c r="B11" s="38">
         <v>1</v>
       </c>
-      <c r="C11" s="29"/>
-      <c r="D11" s="28"/>
-      <c r="E11" s="28"/>
-      <c r="F11" s="31" t="s">
+      <c r="C11" s="39"/>
+      <c r="D11" s="56"/>
+      <c r="E11" s="56"/>
+      <c r="F11" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="G11" s="31" t="s">
+      <c r="G11" s="40" t="s">
         <v>32</v>
       </c>
       <c r="H11" s="25"/>
     </row>
     <row r="12" spans="2:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="34">
+      <c r="B12" s="38">
         <v>2</v>
       </c>
-      <c r="C12" s="29"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="28"/>
-      <c r="F12" s="32"/>
-      <c r="G12" s="32"/>
+      <c r="C12" s="39"/>
+      <c r="D12" s="56"/>
+      <c r="E12" s="56"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="41"/>
       <c r="H12" s="25"/>
     </row>
     <row r="13" spans="2:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="34">
+      <c r="B13" s="38">
         <v>3</v>
       </c>
-      <c r="C13" s="29"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="28"/>
-      <c r="F13" s="32"/>
-      <c r="G13" s="32"/>
+      <c r="C13" s="39"/>
+      <c r="D13" s="56"/>
+      <c r="E13" s="56"/>
+      <c r="F13" s="41"/>
+      <c r="G13" s="41"/>
       <c r="H13" s="25"/>
     </row>
     <row r="14" spans="2:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="34">
+      <c r="B14" s="38">
         <v>4</v>
       </c>
-      <c r="C14" s="29"/>
-      <c r="D14" s="28"/>
-      <c r="E14" s="28"/>
-      <c r="F14" s="32"/>
-      <c r="G14" s="32"/>
+      <c r="C14" s="39"/>
+      <c r="D14" s="56"/>
+      <c r="E14" s="56"/>
+      <c r="F14" s="41"/>
+      <c r="G14" s="41"/>
       <c r="H14" s="25"/>
     </row>
     <row r="15" spans="2:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="34">
+      <c r="B15" s="38">
         <v>5</v>
       </c>
-      <c r="C15" s="29"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="28"/>
-      <c r="F15" s="32"/>
-      <c r="G15" s="32"/>
+      <c r="C15" s="39"/>
+      <c r="D15" s="56"/>
+      <c r="E15" s="56"/>
+      <c r="F15" s="41"/>
+      <c r="G15" s="41"/>
       <c r="H15" s="25"/>
     </row>
     <row r="16" spans="2:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="34">
+      <c r="B16" s="38">
         <v>6</v>
       </c>
-      <c r="C16" s="29"/>
-      <c r="D16" s="28"/>
-      <c r="E16" s="28"/>
-      <c r="F16" s="32"/>
-      <c r="G16" s="32"/>
+      <c r="C16" s="39"/>
+      <c r="D16" s="56"/>
+      <c r="E16" s="56"/>
+      <c r="F16" s="41"/>
+      <c r="G16" s="41"/>
       <c r="H16" s="25"/>
     </row>
     <row r="17" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="34">
+      <c r="B17" s="38">
         <v>7</v>
       </c>
-      <c r="C17" s="29"/>
-      <c r="D17" s="28"/>
-      <c r="E17" s="28"/>
-      <c r="F17" s="32"/>
-      <c r="G17" s="32"/>
+      <c r="C17" s="39"/>
+      <c r="D17" s="56"/>
+      <c r="E17" s="56"/>
+      <c r="F17" s="41"/>
+      <c r="G17" s="41"/>
     </row>
     <row r="18" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="34">
+      <c r="B18" s="38">
         <v>8</v>
       </c>
-      <c r="C18" s="29"/>
-      <c r="D18" s="28"/>
-      <c r="E18" s="28"/>
-      <c r="F18" s="32"/>
-      <c r="G18" s="32"/>
+      <c r="C18" s="39"/>
+      <c r="D18" s="56"/>
+      <c r="E18" s="56"/>
+      <c r="F18" s="41"/>
+      <c r="G18" s="41"/>
     </row>
     <row r="19" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="34">
+      <c r="B19" s="38">
         <v>9</v>
       </c>
-      <c r="C19" s="29"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="28"/>
-      <c r="F19" s="32"/>
-      <c r="G19" s="32"/>
+      <c r="C19" s="39"/>
+      <c r="D19" s="56"/>
+      <c r="E19" s="56"/>
+      <c r="F19" s="41"/>
+      <c r="G19" s="41"/>
     </row>
     <row r="20" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="34">
+      <c r="B20" s="38">
         <v>10</v>
       </c>
-      <c r="C20" s="29"/>
-      <c r="D20" s="28"/>
-      <c r="E20" s="28"/>
-      <c r="F20" s="32"/>
-      <c r="G20" s="32"/>
+      <c r="C20" s="39"/>
+      <c r="D20" s="56"/>
+      <c r="E20" s="56"/>
+      <c r="F20" s="41"/>
+      <c r="G20" s="41"/>
     </row>
     <row r="21" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="34">
+      <c r="B21" s="38">
         <v>11</v>
       </c>
-      <c r="C21" s="29"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="28"/>
-      <c r="F21" s="32"/>
-      <c r="G21" s="32"/>
+      <c r="C21" s="39"/>
+      <c r="D21" s="56"/>
+      <c r="E21" s="56"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="41"/>
     </row>
     <row r="22" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="34">
+      <c r="B22" s="38">
         <v>12</v>
       </c>
-      <c r="C22" s="29"/>
-      <c r="D22" s="28"/>
-      <c r="E22" s="28"/>
-      <c r="F22" s="32"/>
-      <c r="G22" s="32"/>
+      <c r="C22" s="39"/>
+      <c r="D22" s="56"/>
+      <c r="E22" s="56"/>
+      <c r="F22" s="41"/>
+      <c r="G22" s="41"/>
     </row>
     <row r="23" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="34">
+      <c r="B23" s="38">
         <v>13</v>
       </c>
-      <c r="C23" s="29"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="28"/>
-      <c r="F23" s="32"/>
-      <c r="G23" s="32"/>
+      <c r="C23" s="39"/>
+      <c r="D23" s="56"/>
+      <c r="E23" s="56"/>
+      <c r="F23" s="41"/>
+      <c r="G23" s="41"/>
     </row>
     <row r="24" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="34">
+      <c r="B24" s="38">
         <v>14</v>
       </c>
-      <c r="C24" s="29"/>
-      <c r="D24" s="28"/>
-      <c r="E24" s="28"/>
-      <c r="F24" s="32"/>
-      <c r="G24" s="32"/>
+      <c r="C24" s="39"/>
+      <c r="D24" s="56"/>
+      <c r="E24" s="56"/>
+      <c r="F24" s="41"/>
+      <c r="G24" s="41"/>
     </row>
     <row r="25" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="34">
+      <c r="B25" s="38">
         <v>15</v>
       </c>
-      <c r="C25" s="29"/>
-      <c r="D25" s="28"/>
-      <c r="E25" s="28"/>
-      <c r="F25" s="32"/>
-      <c r="G25" s="32"/>
+      <c r="C25" s="39"/>
+      <c r="D25" s="56"/>
+      <c r="E25" s="56"/>
+      <c r="F25" s="41"/>
+      <c r="G25" s="41"/>
     </row>
     <row r="26" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="34">
+      <c r="B26" s="38">
         <v>16</v>
       </c>
-      <c r="C26" s="29"/>
-      <c r="D26" s="28"/>
-      <c r="E26" s="28"/>
-      <c r="F26" s="32"/>
-      <c r="G26" s="32"/>
+      <c r="C26" s="39"/>
+      <c r="D26" s="56"/>
+      <c r="E26" s="56"/>
+      <c r="F26" s="41"/>
+      <c r="G26" s="41"/>
     </row>
     <row r="27" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="34">
+      <c r="B27" s="38">
         <v>17</v>
       </c>
-      <c r="C27" s="29"/>
-      <c r="D27" s="28"/>
-      <c r="E27" s="28"/>
-      <c r="F27" s="32"/>
-      <c r="G27" s="32"/>
+      <c r="C27" s="39"/>
+      <c r="D27" s="56"/>
+      <c r="E27" s="56"/>
+      <c r="F27" s="41"/>
+      <c r="G27" s="41"/>
     </row>
     <row r="28" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="34">
+      <c r="B28" s="38">
         <v>18</v>
       </c>
-      <c r="C28" s="29"/>
-      <c r="D28" s="28"/>
-      <c r="E28" s="28"/>
-      <c r="F28" s="32"/>
-      <c r="G28" s="32"/>
+      <c r="C28" s="39"/>
+      <c r="D28" s="56"/>
+      <c r="E28" s="56"/>
+      <c r="F28" s="41"/>
+      <c r="G28" s="41"/>
     </row>
     <row r="29" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="34">
+      <c r="B29" s="38">
         <v>19</v>
       </c>
-      <c r="C29" s="29"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="28"/>
-      <c r="F29" s="32"/>
-      <c r="G29" s="32"/>
+      <c r="C29" s="39"/>
+      <c r="D29" s="56"/>
+      <c r="E29" s="56"/>
+      <c r="F29" s="41"/>
+      <c r="G29" s="41"/>
     </row>
     <row r="30" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="34">
+      <c r="B30" s="38">
         <v>20</v>
       </c>
-      <c r="C30" s="29"/>
-      <c r="D30" s="28"/>
-      <c r="E30" s="28"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="32"/>
+      <c r="C30" s="39"/>
+      <c r="D30" s="56"/>
+      <c r="E30" s="56"/>
+      <c r="F30" s="41"/>
+      <c r="G30" s="41"/>
     </row>
     <row r="31" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="34">
+      <c r="B31" s="38">
         <v>21</v>
       </c>
-      <c r="C31" s="29"/>
-      <c r="D31" s="28"/>
-      <c r="E31" s="28"/>
-      <c r="F31" s="32"/>
-      <c r="G31" s="32"/>
+      <c r="C31" s="39"/>
+      <c r="D31" s="56"/>
+      <c r="E31" s="56"/>
+      <c r="F31" s="41"/>
+      <c r="G31" s="41"/>
     </row>
     <row r="32" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="34">
+      <c r="B32" s="38">
         <v>22</v>
       </c>
-      <c r="C32" s="29"/>
-      <c r="D32" s="28"/>
-      <c r="E32" s="28"/>
-      <c r="F32" s="32"/>
-      <c r="G32" s="32"/>
+      <c r="C32" s="39"/>
+      <c r="D32" s="56"/>
+      <c r="E32" s="56"/>
+      <c r="F32" s="41"/>
+      <c r="G32" s="41"/>
     </row>
     <row r="33" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="34">
+      <c r="B33" s="38">
         <v>23</v>
       </c>
-      <c r="C33" s="29"/>
-      <c r="D33" s="28"/>
-      <c r="E33" s="28"/>
-      <c r="F33" s="32"/>
-      <c r="G33" s="32"/>
+      <c r="C33" s="39"/>
+      <c r="D33" s="56"/>
+      <c r="E33" s="56"/>
+      <c r="F33" s="41"/>
+      <c r="G33" s="41"/>
     </row>
     <row r="34" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="34">
+      <c r="B34" s="38">
         <v>24</v>
       </c>
-      <c r="C34" s="29"/>
-      <c r="D34" s="28"/>
-      <c r="E34" s="28"/>
-      <c r="F34" s="32"/>
-      <c r="G34" s="32"/>
+      <c r="C34" s="39"/>
+      <c r="D34" s="56"/>
+      <c r="E34" s="56"/>
+      <c r="F34" s="41"/>
+      <c r="G34" s="41"/>
     </row>
     <row r="35" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="34">
+      <c r="B35" s="38">
         <v>25</v>
       </c>
-      <c r="C35" s="29"/>
-      <c r="D35" s="28"/>
-      <c r="E35" s="28"/>
-      <c r="F35" s="32"/>
-      <c r="G35" s="32"/>
+      <c r="C35" s="39"/>
+      <c r="D35" s="56"/>
+      <c r="E35" s="56"/>
+      <c r="F35" s="41"/>
+      <c r="G35" s="41"/>
     </row>
     <row r="36" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="34">
+      <c r="B36" s="38">
         <v>26</v>
       </c>
-      <c r="C36" s="29"/>
-      <c r="D36" s="28"/>
-      <c r="E36" s="28"/>
-      <c r="F36" s="32"/>
-      <c r="G36" s="32"/>
+      <c r="C36" s="39"/>
+      <c r="D36" s="56"/>
+      <c r="E36" s="56"/>
+      <c r="F36" s="41"/>
+      <c r="G36" s="41"/>
     </row>
     <row r="37" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="34">
+      <c r="B37" s="38">
         <v>27</v>
       </c>
-      <c r="C37" s="29"/>
-      <c r="D37" s="28"/>
-      <c r="E37" s="28"/>
-      <c r="F37" s="32"/>
-      <c r="G37" s="32"/>
+      <c r="C37" s="39"/>
+      <c r="D37" s="56"/>
+      <c r="E37" s="56"/>
+      <c r="F37" s="41"/>
+      <c r="G37" s="41"/>
     </row>
     <row r="38" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="34">
+      <c r="B38" s="38">
         <v>28</v>
       </c>
-      <c r="C38" s="29"/>
-      <c r="D38" s="28"/>
-      <c r="E38" s="28"/>
-      <c r="F38" s="32"/>
-      <c r="G38" s="32"/>
+      <c r="C38" s="39"/>
+      <c r="D38" s="56"/>
+      <c r="E38" s="56"/>
+      <c r="F38" s="41"/>
+      <c r="G38" s="41"/>
     </row>
     <row r="39" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="34">
+      <c r="B39" s="38">
         <v>29</v>
       </c>
-      <c r="C39" s="29"/>
-      <c r="D39" s="28"/>
-      <c r="E39" s="28"/>
-      <c r="F39" s="32"/>
-      <c r="G39" s="32"/>
+      <c r="C39" s="39"/>
+      <c r="D39" s="56"/>
+      <c r="E39" s="56"/>
+      <c r="F39" s="41"/>
+      <c r="G39" s="41"/>
     </row>
     <row r="40" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="34">
+      <c r="B40" s="38">
         <v>30</v>
       </c>
-      <c r="C40" s="29"/>
-      <c r="D40" s="28"/>
-      <c r="E40" s="28"/>
-      <c r="F40" s="32"/>
-      <c r="G40" s="32"/>
+      <c r="C40" s="39"/>
+      <c r="D40" s="56"/>
+      <c r="E40" s="56"/>
+      <c r="F40" s="41"/>
+      <c r="G40" s="41"/>
     </row>
     <row r="41" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="34">
+      <c r="B41" s="38">
         <v>31</v>
       </c>
-      <c r="C41" s="29"/>
-      <c r="D41" s="28"/>
-      <c r="E41" s="28"/>
-      <c r="F41" s="32"/>
-      <c r="G41" s="32"/>
+      <c r="C41" s="39"/>
+      <c r="D41" s="56"/>
+      <c r="E41" s="56"/>
+      <c r="F41" s="41"/>
+      <c r="G41" s="41"/>
     </row>
     <row r="42" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="34">
+      <c r="B42" s="38">
         <v>32</v>
       </c>
-      <c r="C42" s="29"/>
-      <c r="D42" s="28"/>
-      <c r="E42" s="28"/>
-      <c r="F42" s="32"/>
-      <c r="G42" s="32"/>
+      <c r="C42" s="39"/>
+      <c r="D42" s="56"/>
+      <c r="E42" s="56"/>
+      <c r="F42" s="41"/>
+      <c r="G42" s="41"/>
     </row>
     <row r="43" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="34">
+      <c r="B43" s="38">
         <v>33</v>
       </c>
-      <c r="C43" s="29"/>
-      <c r="D43" s="28"/>
-      <c r="E43" s="28"/>
-      <c r="F43" s="32"/>
-      <c r="G43" s="32"/>
+      <c r="C43" s="39"/>
+      <c r="D43" s="56"/>
+      <c r="E43" s="56"/>
+      <c r="F43" s="41"/>
+      <c r="G43" s="41"/>
     </row>
     <row r="44" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="34">
+      <c r="B44" s="38">
         <v>34</v>
       </c>
-      <c r="C44" s="29"/>
-      <c r="D44" s="28"/>
-      <c r="E44" s="28"/>
-      <c r="F44" s="32"/>
-      <c r="G44" s="32"/>
+      <c r="C44" s="39"/>
+      <c r="D44" s="56"/>
+      <c r="E44" s="56"/>
+      <c r="F44" s="41"/>
+      <c r="G44" s="41"/>
     </row>
     <row r="45" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="34">
+      <c r="B45" s="38">
         <v>35</v>
       </c>
-      <c r="C45" s="29"/>
-      <c r="D45" s="28"/>
-      <c r="E45" s="28"/>
-      <c r="F45" s="32"/>
-      <c r="G45" s="32"/>
+      <c r="C45" s="39"/>
+      <c r="D45" s="56"/>
+      <c r="E45" s="56"/>
+      <c r="F45" s="41"/>
+      <c r="G45" s="41"/>
     </row>
     <row r="46" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="34">
+      <c r="B46" s="38">
         <v>36</v>
       </c>
-      <c r="C46" s="29"/>
-      <c r="D46" s="28"/>
-      <c r="E46" s="28"/>
-      <c r="F46" s="32"/>
-      <c r="G46" s="32"/>
+      <c r="C46" s="39"/>
+      <c r="D46" s="56"/>
+      <c r="E46" s="56"/>
+      <c r="F46" s="41"/>
+      <c r="G46" s="41"/>
     </row>
     <row r="47" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="34">
+      <c r="B47" s="38">
         <v>37</v>
       </c>
-      <c r="C47" s="29"/>
-      <c r="D47" s="28"/>
-      <c r="E47" s="28"/>
-      <c r="F47" s="32"/>
-      <c r="G47" s="32"/>
+      <c r="C47" s="39"/>
+      <c r="D47" s="56"/>
+      <c r="E47" s="56"/>
+      <c r="F47" s="41"/>
+      <c r="G47" s="41"/>
     </row>
     <row r="48" spans="2:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="34">
+      <c r="B48" s="38">
         <v>38</v>
       </c>
-      <c r="C48" s="29"/>
-      <c r="D48" s="28"/>
-      <c r="E48" s="28"/>
-      <c r="F48" s="32"/>
-      <c r="G48" s="32"/>
+      <c r="C48" s="39"/>
+      <c r="D48" s="56"/>
+      <c r="E48" s="56"/>
+      <c r="F48" s="41"/>
+      <c r="G48" s="41"/>
     </row>
     <row r="49" spans="2:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="34">
+      <c r="B49" s="38">
         <v>39</v>
       </c>
-      <c r="C49" s="29"/>
-      <c r="D49" s="28"/>
-      <c r="E49" s="28"/>
-      <c r="F49" s="32"/>
-      <c r="G49" s="32"/>
+      <c r="C49" s="39"/>
+      <c r="D49" s="56"/>
+      <c r="E49" s="56"/>
+      <c r="F49" s="41"/>
+      <c r="G49" s="41"/>
     </row>
     <row r="50" spans="2:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="34">
+      <c r="B50" s="38">
         <v>40</v>
       </c>
-      <c r="C50" s="29"/>
-      <c r="D50" s="28"/>
-      <c r="E50" s="28"/>
-      <c r="F50" s="32"/>
-      <c r="G50" s="32"/>
+      <c r="C50" s="39"/>
+      <c r="D50" s="56"/>
+      <c r="E50" s="56"/>
+      <c r="F50" s="41"/>
+      <c r="G50" s="41"/>
     </row>
     <row r="51" spans="2:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="34">
+      <c r="B51" s="38">
         <v>41</v>
       </c>
-      <c r="C51" s="29"/>
-      <c r="D51" s="28"/>
-      <c r="E51" s="28"/>
-      <c r="F51" s="32"/>
-      <c r="G51" s="32"/>
+      <c r="C51" s="39"/>
+      <c r="D51" s="56"/>
+      <c r="E51" s="56"/>
+      <c r="F51" s="41"/>
+      <c r="G51" s="41"/>
     </row>
     <row r="52" spans="2:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="34">
+      <c r="B52" s="38">
         <v>42</v>
       </c>
-      <c r="C52" s="29"/>
-      <c r="D52" s="28"/>
-      <c r="E52" s="28"/>
-      <c r="F52" s="32"/>
-      <c r="G52" s="32"/>
+      <c r="C52" s="39"/>
+      <c r="D52" s="56"/>
+      <c r="E52" s="56"/>
+      <c r="F52" s="41"/>
+      <c r="G52" s="41"/>
     </row>
     <row r="53" spans="2:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="34">
+      <c r="B53" s="38">
         <v>43</v>
       </c>
-      <c r="C53" s="29"/>
-      <c r="D53" s="28"/>
-      <c r="E53" s="28"/>
-      <c r="F53" s="32"/>
-      <c r="G53" s="32"/>
+      <c r="C53" s="39"/>
+      <c r="D53" s="56"/>
+      <c r="E53" s="56"/>
+      <c r="F53" s="41"/>
+      <c r="G53" s="41"/>
     </row>
     <row r="54" spans="2:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="34">
+      <c r="B54" s="38">
         <v>44</v>
       </c>
-      <c r="C54" s="29"/>
-      <c r="D54" s="28"/>
-      <c r="E54" s="28"/>
-      <c r="F54" s="32"/>
-      <c r="G54" s="32"/>
+      <c r="C54" s="39"/>
+      <c r="D54" s="56"/>
+      <c r="E54" s="56"/>
+      <c r="F54" s="41"/>
+      <c r="G54" s="41"/>
     </row>
     <row r="55" spans="2:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="34">
+      <c r="B55" s="38">
         <v>45</v>
       </c>
-      <c r="C55" s="34"/>
-      <c r="D55" s="28"/>
-      <c r="E55" s="28"/>
-      <c r="F55" s="33"/>
-      <c r="G55" s="33"/>
+      <c r="C55" s="38"/>
+      <c r="D55" s="56"/>
+      <c r="E55" s="56"/>
+      <c r="F55" s="42"/>
+      <c r="G55" s="42"/>
     </row>
     <row r="62" spans="2:8" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="40"/>
-      <c r="C62" s="41"/>
-      <c r="D62" s="42"/>
-      <c r="E62" s="42"/>
-      <c r="F62" s="42"/>
-      <c r="G62" s="42"/>
+      <c r="B62" s="31"/>
+      <c r="C62" s="32"/>
+      <c r="D62" s="33"/>
+      <c r="E62" s="33"/>
+      <c r="F62" s="33"/>
+      <c r="G62" s="33"/>
     </row>
     <row r="63" spans="2:8" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B63" s="43" t="s">
@@ -2578,36 +2577,36 @@
       <c r="H63" s="25"/>
     </row>
     <row r="64" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B64" s="35" t="s">
+      <c r="B64" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="C64" s="36"/>
-      <c r="D64" s="39" t="s">
+      <c r="C64" s="47"/>
+      <c r="D64" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="E64" s="39"/>
-      <c r="F64" s="39" t="s">
+      <c r="E64" s="50"/>
+      <c r="F64" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="G64" s="39"/>
+      <c r="G64" s="50"/>
       <c r="H64" s="25"/>
     </row>
     <row r="65" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B65" s="35"/>
-      <c r="C65" s="36"/>
-      <c r="D65" s="39" t="s">
+      <c r="B65" s="46"/>
+      <c r="C65" s="47"/>
+      <c r="D65" s="50" t="s">
         <v>31</v>
       </c>
-      <c r="E65" s="39"/>
-      <c r="F65" s="39" t="s">
+      <c r="E65" s="50"/>
+      <c r="F65" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="G65" s="39"/>
+      <c r="G65" s="50"/>
       <c r="H65" s="25"/>
     </row>
     <row r="66" spans="2:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B66" s="37"/>
-      <c r="C66" s="38"/>
+      <c r="B66" s="48"/>
+      <c r="C66" s="49"/>
       <c r="D66" s="26" t="s">
         <v>29</v>
       </c>
@@ -2623,59 +2622,90 @@
       <c r="H66" s="25"/>
     </row>
     <row r="67" spans="2:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B67" s="29">
+      <c r="B67" s="39">
         <v>46</v>
       </c>
-      <c r="C67" s="30"/>
-      <c r="D67" s="28"/>
-      <c r="E67" s="28"/>
-      <c r="F67" s="31" t="s">
+      <c r="C67" s="51"/>
+      <c r="D67" s="56"/>
+      <c r="E67" s="56"/>
+      <c r="F67" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="G67" s="31" t="s">
+      <c r="G67" s="40" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="68" spans="2:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B68" s="34">
+      <c r="B68" s="38">
         <v>47</v>
       </c>
-      <c r="C68" s="29"/>
-      <c r="D68" s="28"/>
-      <c r="E68" s="28"/>
-      <c r="F68" s="32"/>
-      <c r="G68" s="32"/>
+      <c r="C68" s="39"/>
+      <c r="D68" s="56"/>
+      <c r="E68" s="56"/>
+      <c r="F68" s="41"/>
+      <c r="G68" s="41"/>
     </row>
     <row r="69" spans="2:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B69" s="34">
+      <c r="B69" s="38">
         <v>48</v>
       </c>
-      <c r="C69" s="29"/>
-      <c r="D69" s="28"/>
-      <c r="E69" s="28"/>
-      <c r="F69" s="33"/>
-      <c r="G69" s="33"/>
+      <c r="C69" s="39"/>
+      <c r="D69" s="56"/>
+      <c r="E69" s="56"/>
+      <c r="F69" s="42"/>
+      <c r="G69" s="42"/>
     </row>
     <row r="72" spans="2:8" x14ac:dyDescent="0.25">
       <c r="E72"/>
     </row>
   </sheetData>
   <mergeCells count="77">
-    <mergeCell ref="B1:G1"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="D6:G6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="B8:C10"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="B67:C67"/>
+    <mergeCell ref="F67:F69"/>
+    <mergeCell ref="G67:G69"/>
+    <mergeCell ref="B68:C68"/>
+    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="B64:C66"/>
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="F64:G64"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="F65:G65"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="D62:G62"/>
+    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="D63:E63"/>
+    <mergeCell ref="F63:G63"/>
+    <mergeCell ref="B50:C50"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:C29"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="F11:F55"/>
     <mergeCell ref="G11:G55"/>
@@ -2692,52 +2722,21 @@
     <mergeCell ref="B22:C22"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="B49:C49"/>
-    <mergeCell ref="B50:C50"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="D62:G62"/>
-    <mergeCell ref="B63:C63"/>
-    <mergeCell ref="D63:E63"/>
-    <mergeCell ref="F63:G63"/>
-    <mergeCell ref="B64:C66"/>
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="F64:G64"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="F65:G65"/>
-    <mergeCell ref="B67:C67"/>
-    <mergeCell ref="F67:F69"/>
-    <mergeCell ref="G67:G69"/>
-    <mergeCell ref="B68:C68"/>
-    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="B8:C10"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="D6:G6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="B1:G1"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D4:E4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>